<commit_message>
Add file train h5
</commit_message>
<xml_diff>
--- a/ai/data/metadata.xlsx
+++ b/ai/data/metadata.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NCKH\CNN_dog_cat\training\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\NCKH_Web\PetAI\ai\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A451E780-EBC7-45C9-AE81-552056DF08C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="11472"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="11472" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="661">
   <si>
     <t>STT</t>
   </si>
@@ -2777,11 +2767,14 @@
 Về vận động, Burmese khá hiếu động và thích chơi đùa, leo trèo. Chủ nuôi nên chuẩn bị đồ chơi, trụ cào móng hoặc không gian leo trèo trong nhà để giúp mèo giải tỏa năng lượng và tránh buồn chán. Chúng thích ở trong nhà và không cần ra ngoài thường xuyên như một số giống mèo khác.
 Về sức khỏe, Burmese nhìn chung khỏe mạnh nhưng có thể gặp một số vấn đề di truyền như bệnh nướu răng hoặc bệnh tim nhẹ. Việc vệ sinh răng miệng định kỳ, khám thú y thường xuyên và tiêm phòng đầy đủ là rất quan trọng. Tính cách của Burmese rất tình cảm, hòa đồng với trẻ em và các vật nuôi khác, phù hợp với gia đình cần một giống mèo thân thiện, gắn bó và dễ chăm sóc.</t>
   </si>
+  <si>
+    <t>unknown</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -3160,12 +3153,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P141"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:P142"/>
   <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="4.296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="5.296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.09765625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.09765625" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.69921875" style="1" customWidth="1"/>
     <col min="5" max="16384" width="9.09765625" style="1"/>
@@ -8121,6 +8114,17 @@
         <v>658</v>
       </c>
     </row>
+    <row r="142" spans="1:11">
+      <c r="A142" s="1">
+        <v>140</v>
+      </c>
+      <c r="B142" t="s">
+        <v>660</v>
+      </c>
+      <c r="C142" t="s">
+        <v>660</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>